<commit_message>
etsy: novo visual sem cara de IA (fundo branco, fotos com notebook e close legivel) e estoque revisado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DYz1Azd3FHBSgFnLhXfMUY
</commit_message>
<xml_diff>
--- a/etsy/inventory/Inventory-Sales-Tracker.xlsx
+++ b/etsy/inventory/Inventory-Sales-Tracker.xlsx
@@ -96,7 +96,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -105,8 +105,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F6F4EF"/>
-        <bgColor rgb="00F6F4EF"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,12 +119,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF4C2"/>
         <bgColor rgb="00FFF4C2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -168,16 +162,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D4C7"/>
+        <color rgb="00D5DBDB"/>
       </bottom>
     </border>
   </borders>
@@ -195,31 +189,33 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="8" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -228,13 +224,13 @@
     <xf numFmtId="1" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -780,7 +776,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Your shop at a glance</t>
+          <t>Shop dashboard</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -799,7 +795,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Pick the month and year. Stock is always 'now'.</t>
+          <t>Pick a month and a year. Stock figures are always as of today.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -909,7 +905,7 @@
       </c>
       <c r="G7" s="1" t="n"/>
       <c r="H7" s="13">
-        <f>COUNTIFS(Products!$M$6:$M$205,"⚠*")+COUNTIFS(Products!$M$6:$M$205,"✗*")</f>
+        <f>COUNTIFS(Products!$M$6:$M$205,"Reorder now")+COUNTIFS(Products!$M$6:$M$205,"Out of stock")</f>
         <v/>
       </c>
       <c r="I7" s="1" t="n"/>
@@ -978,7 +974,7 @@
       <c r="F10" s="1" t="n"/>
       <c r="G10" s="1" t="n"/>
       <c r="H10" s="19">
-        <f>COUNTIFS(Products!$M$6:$M$205,"✗*")&amp;" product(s) out of stock"</f>
+        <f>IF(COUNTIFS(Products!$M$6:$M$205,"Out of stock")=0,"Nothing is out of stock",IF(COUNTIFS(Products!$M$6:$M$205,"Out of stock")=1,"1 product is out of stock",COUNTIFS(Products!$M$6:$M$205,"Out of stock")&amp;" products are out of stock"))</f>
         <v/>
       </c>
       <c r="I10" s="1" t="n"/>
@@ -1005,7 +1001,7 @@
       <c r="F11" s="1" t="n"/>
       <c r="G11" s="1" t="n"/>
       <c r="H11" s="20">
-        <f>COUNTIFS(Products!$M$6:$M$205,"⚠*")&amp;" product(s) at or below the reorder level"</f>
+        <f>IF(COUNTIFS(Products!$M$6:$M$205,"Reorder now")=0,"No product is at its reorder level",IF(COUNTIFS(Products!$M$6:$M$205,"Reorder now")=1,"1 product is at its reorder level",COUNTIFS(Products!$M$6:$M$205,"Reorder now")&amp;" products are at their reorder level"))</f>
         <v/>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -1032,7 +1028,7 @@
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
       <c r="H12" s="21">
-        <f>"Best seller (all time): "&amp;IFERROR(INDEX(Products!$C$6:$C$205,MATCH(MAX(Products!$J$6:$J$205),Products!$J$6:$J$205,0)),"—")</f>
+        <f>"Best seller so far: "&amp;IFERROR(INDEX(Products!$C$6:$C$205,MATCH(MAX(Products!$J$6:$J$205),Products!$J$6:$J$205,0)),"none yet")</f>
         <v/>
       </c>
       <c r="I12" s="1" t="n"/>
@@ -1059,7 +1055,7 @@
       <c r="F13" s="1" t="n"/>
       <c r="G13" s="1" t="n"/>
       <c r="H13" s="22">
-        <f>"Average margin: "&amp;IFERROR(FIXED(AVERAGE(Products!$L$6:$L$205)*100,0)&amp;"%","—")</f>
+        <f>"Average margin: "&amp;IFERROR(FIXED(AVERAGE(Products!$L$6:$L$205)*100,0)&amp;"%","n/a")</f>
         <v/>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -1895,8 +1891,13 @@
       <c r="I79" s="1" t="n"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="H10:H11">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LEFT(H10,2)="No"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B10:E21">
-    <cfRule type="expression" priority="1" dxfId="0">
+    <cfRule type="expression" priority="2" dxfId="0">
       <formula>ROW()-9=$J$1</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2117,7 +2118,7 @@
         <v/>
       </c>
       <c r="M6" s="29">
-        <f>IF(B6="","",IF(K6&lt;=0,"✗ Out of stock",IF(K6&lt;=H6,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B6="","",IF(K6&lt;=0,"Out of stock",IF(K6&lt;=H6,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N6" s="1" t="n"/>
@@ -2168,7 +2169,7 @@
         <v/>
       </c>
       <c r="M7" s="29">
-        <f>IF(B7="","",IF(K7&lt;=0,"✗ Out of stock",IF(K7&lt;=H7,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B7="","",IF(K7&lt;=0,"Out of stock",IF(K7&lt;=H7,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N7" s="1" t="n"/>
@@ -2219,7 +2220,7 @@
         <v/>
       </c>
       <c r="M8" s="29">
-        <f>IF(B8="","",IF(K8&lt;=0,"✗ Out of stock",IF(K8&lt;=H8,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B8="","",IF(K8&lt;=0,"Out of stock",IF(K8&lt;=H8,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N8" s="1" t="n"/>
@@ -2251,7 +2252,7 @@
         <v>30</v>
       </c>
       <c r="H9" s="26" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I9" s="18">
         <f>IF(B9="","",SUMIFS('Stock Moves'!$E$6:$E$2005,'Stock Moves'!$C$6:$C$2005,B9,'Stock Moves'!$D$6:$D$2005,"Purchase")+SUMIFS('Stock Moves'!$E$6:$E$2005,'Stock Moves'!$C$6:$C$2005,B9,'Stock Moves'!$D$6:$D$2005,"Return")+SUMIFS('Stock Moves'!$E$6:$E$2005,'Stock Moves'!$C$6:$C$2005,B9,'Stock Moves'!$D$6:$D$2005,"Adjustment"))</f>
@@ -2270,7 +2271,7 @@
         <v/>
       </c>
       <c r="M9" s="29">
-        <f>IF(B9="","",IF(K9&lt;=0,"✗ Out of stock",IF(K9&lt;=H9,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B9="","",IF(K9&lt;=0,"Out of stock",IF(K9&lt;=H9,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N9" s="1" t="n"/>
@@ -2302,7 +2303,7 @@
         <v>40</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="I10" s="18">
         <f>IF(B10="","",SUMIFS('Stock Moves'!$E$6:$E$2005,'Stock Moves'!$C$6:$C$2005,B10,'Stock Moves'!$D$6:$D$2005,"Purchase")+SUMIFS('Stock Moves'!$E$6:$E$2005,'Stock Moves'!$C$6:$C$2005,B10,'Stock Moves'!$D$6:$D$2005,"Return")+SUMIFS('Stock Moves'!$E$6:$E$2005,'Stock Moves'!$C$6:$C$2005,B10,'Stock Moves'!$D$6:$D$2005,"Adjustment"))</f>
@@ -2321,7 +2322,7 @@
         <v/>
       </c>
       <c r="M10" s="29">
-        <f>IF(B10="","",IF(K10&lt;=0,"✗ Out of stock",IF(K10&lt;=H10,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B10="","",IF(K10&lt;=0,"Out of stock",IF(K10&lt;=H10,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N10" s="1" t="n"/>
@@ -2372,7 +2373,7 @@
         <v/>
       </c>
       <c r="M11" s="29">
-        <f>IF(B11="","",IF(K11&lt;=0,"✗ Out of stock",IF(K11&lt;=H11,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B11="","",IF(K11&lt;=0,"Out of stock",IF(K11&lt;=H11,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N11" s="1" t="n"/>
@@ -2403,7 +2404,7 @@
         <v/>
       </c>
       <c r="M12" s="29">
-        <f>IF(B12="","",IF(K12&lt;=0,"✗ Out of stock",IF(K12&lt;=H12,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B12="","",IF(K12&lt;=0,"Out of stock",IF(K12&lt;=H12,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N12" s="1" t="n"/>
@@ -2434,7 +2435,7 @@
         <v/>
       </c>
       <c r="M13" s="29">
-        <f>IF(B13="","",IF(K13&lt;=0,"✗ Out of stock",IF(K13&lt;=H13,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B13="","",IF(K13&lt;=0,"Out of stock",IF(K13&lt;=H13,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N13" s="1" t="n"/>
@@ -2465,7 +2466,7 @@
         <v/>
       </c>
       <c r="M14" s="29">
-        <f>IF(B14="","",IF(K14&lt;=0,"✗ Out of stock",IF(K14&lt;=H14,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B14="","",IF(K14&lt;=0,"Out of stock",IF(K14&lt;=H14,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N14" s="1" t="n"/>
@@ -2496,7 +2497,7 @@
         <v/>
       </c>
       <c r="M15" s="29">
-        <f>IF(B15="","",IF(K15&lt;=0,"✗ Out of stock",IF(K15&lt;=H15,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B15="","",IF(K15&lt;=0,"Out of stock",IF(K15&lt;=H15,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N15" s="1" t="n"/>
@@ -2527,7 +2528,7 @@
         <v/>
       </c>
       <c r="M16" s="29">
-        <f>IF(B16="","",IF(K16&lt;=0,"✗ Out of stock",IF(K16&lt;=H16,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B16="","",IF(K16&lt;=0,"Out of stock",IF(K16&lt;=H16,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N16" s="1" t="n"/>
@@ -2558,7 +2559,7 @@
         <v/>
       </c>
       <c r="M17" s="29">
-        <f>IF(B17="","",IF(K17&lt;=0,"✗ Out of stock",IF(K17&lt;=H17,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B17="","",IF(K17&lt;=0,"Out of stock",IF(K17&lt;=H17,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N17" s="1" t="n"/>
@@ -2589,7 +2590,7 @@
         <v/>
       </c>
       <c r="M18" s="29">
-        <f>IF(B18="","",IF(K18&lt;=0,"✗ Out of stock",IF(K18&lt;=H18,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B18="","",IF(K18&lt;=0,"Out of stock",IF(K18&lt;=H18,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N18" s="1" t="n"/>
@@ -2620,7 +2621,7 @@
         <v/>
       </c>
       <c r="M19" s="29">
-        <f>IF(B19="","",IF(K19&lt;=0,"✗ Out of stock",IF(K19&lt;=H19,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B19="","",IF(K19&lt;=0,"Out of stock",IF(K19&lt;=H19,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N19" s="1" t="n"/>
@@ -2651,7 +2652,7 @@
         <v/>
       </c>
       <c r="M20" s="29">
-        <f>IF(B20="","",IF(K20&lt;=0,"✗ Out of stock",IF(K20&lt;=H20,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B20="","",IF(K20&lt;=0,"Out of stock",IF(K20&lt;=H20,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N20" s="1" t="n"/>
@@ -2682,7 +2683,7 @@
         <v/>
       </c>
       <c r="M21" s="29">
-        <f>IF(B21="","",IF(K21&lt;=0,"✗ Out of stock",IF(K21&lt;=H21,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B21="","",IF(K21&lt;=0,"Out of stock",IF(K21&lt;=H21,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N21" s="1" t="n"/>
@@ -2713,7 +2714,7 @@
         <v/>
       </c>
       <c r="M22" s="29">
-        <f>IF(B22="","",IF(K22&lt;=0,"✗ Out of stock",IF(K22&lt;=H22,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B22="","",IF(K22&lt;=0,"Out of stock",IF(K22&lt;=H22,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N22" s="1" t="n"/>
@@ -2744,7 +2745,7 @@
         <v/>
       </c>
       <c r="M23" s="29">
-        <f>IF(B23="","",IF(K23&lt;=0,"✗ Out of stock",IF(K23&lt;=H23,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B23="","",IF(K23&lt;=0,"Out of stock",IF(K23&lt;=H23,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N23" s="1" t="n"/>
@@ -2775,7 +2776,7 @@
         <v/>
       </c>
       <c r="M24" s="29">
-        <f>IF(B24="","",IF(K24&lt;=0,"✗ Out of stock",IF(K24&lt;=H24,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B24="","",IF(K24&lt;=0,"Out of stock",IF(K24&lt;=H24,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N24" s="1" t="n"/>
@@ -2806,7 +2807,7 @@
         <v/>
       </c>
       <c r="M25" s="29">
-        <f>IF(B25="","",IF(K25&lt;=0,"✗ Out of stock",IF(K25&lt;=H25,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B25="","",IF(K25&lt;=0,"Out of stock",IF(K25&lt;=H25,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N25" s="1" t="n"/>
@@ -2837,7 +2838,7 @@
         <v/>
       </c>
       <c r="M26" s="29">
-        <f>IF(B26="","",IF(K26&lt;=0,"✗ Out of stock",IF(K26&lt;=H26,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B26="","",IF(K26&lt;=0,"Out of stock",IF(K26&lt;=H26,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N26" s="1" t="n"/>
@@ -2868,7 +2869,7 @@
         <v/>
       </c>
       <c r="M27" s="29">
-        <f>IF(B27="","",IF(K27&lt;=0,"✗ Out of stock",IF(K27&lt;=H27,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B27="","",IF(K27&lt;=0,"Out of stock",IF(K27&lt;=H27,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N27" s="1" t="n"/>
@@ -2899,7 +2900,7 @@
         <v/>
       </c>
       <c r="M28" s="29">
-        <f>IF(B28="","",IF(K28&lt;=0,"✗ Out of stock",IF(K28&lt;=H28,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B28="","",IF(K28&lt;=0,"Out of stock",IF(K28&lt;=H28,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N28" s="1" t="n"/>
@@ -2930,7 +2931,7 @@
         <v/>
       </c>
       <c r="M29" s="29">
-        <f>IF(B29="","",IF(K29&lt;=0,"✗ Out of stock",IF(K29&lt;=H29,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B29="","",IF(K29&lt;=0,"Out of stock",IF(K29&lt;=H29,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N29" s="1" t="n"/>
@@ -2961,7 +2962,7 @@
         <v/>
       </c>
       <c r="M30" s="29">
-        <f>IF(B30="","",IF(K30&lt;=0,"✗ Out of stock",IF(K30&lt;=H30,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B30="","",IF(K30&lt;=0,"Out of stock",IF(K30&lt;=H30,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N30" s="1" t="n"/>
@@ -2992,7 +2993,7 @@
         <v/>
       </c>
       <c r="M31" s="29">
-        <f>IF(B31="","",IF(K31&lt;=0,"✗ Out of stock",IF(K31&lt;=H31,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B31="","",IF(K31&lt;=0,"Out of stock",IF(K31&lt;=H31,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N31" s="1" t="n"/>
@@ -3023,7 +3024,7 @@
         <v/>
       </c>
       <c r="M32" s="29">
-        <f>IF(B32="","",IF(K32&lt;=0,"✗ Out of stock",IF(K32&lt;=H32,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B32="","",IF(K32&lt;=0,"Out of stock",IF(K32&lt;=H32,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N32" s="1" t="n"/>
@@ -3054,7 +3055,7 @@
         <v/>
       </c>
       <c r="M33" s="29">
-        <f>IF(B33="","",IF(K33&lt;=0,"✗ Out of stock",IF(K33&lt;=H33,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B33="","",IF(K33&lt;=0,"Out of stock",IF(K33&lt;=H33,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N33" s="1" t="n"/>
@@ -3085,7 +3086,7 @@
         <v/>
       </c>
       <c r="M34" s="29">
-        <f>IF(B34="","",IF(K34&lt;=0,"✗ Out of stock",IF(K34&lt;=H34,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B34="","",IF(K34&lt;=0,"Out of stock",IF(K34&lt;=H34,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N34" s="1" t="n"/>
@@ -3116,7 +3117,7 @@
         <v/>
       </c>
       <c r="M35" s="29">
-        <f>IF(B35="","",IF(K35&lt;=0,"✗ Out of stock",IF(K35&lt;=H35,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B35="","",IF(K35&lt;=0,"Out of stock",IF(K35&lt;=H35,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N35" s="1" t="n"/>
@@ -3147,7 +3148,7 @@
         <v/>
       </c>
       <c r="M36" s="29">
-        <f>IF(B36="","",IF(K36&lt;=0,"✗ Out of stock",IF(K36&lt;=H36,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B36="","",IF(K36&lt;=0,"Out of stock",IF(K36&lt;=H36,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N36" s="1" t="n"/>
@@ -3178,7 +3179,7 @@
         <v/>
       </c>
       <c r="M37" s="29">
-        <f>IF(B37="","",IF(K37&lt;=0,"✗ Out of stock",IF(K37&lt;=H37,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B37="","",IF(K37&lt;=0,"Out of stock",IF(K37&lt;=H37,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N37" s="1" t="n"/>
@@ -3209,7 +3210,7 @@
         <v/>
       </c>
       <c r="M38" s="29">
-        <f>IF(B38="","",IF(K38&lt;=0,"✗ Out of stock",IF(K38&lt;=H38,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B38="","",IF(K38&lt;=0,"Out of stock",IF(K38&lt;=H38,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N38" s="1" t="n"/>
@@ -3240,7 +3241,7 @@
         <v/>
       </c>
       <c r="M39" s="29">
-        <f>IF(B39="","",IF(K39&lt;=0,"✗ Out of stock",IF(K39&lt;=H39,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B39="","",IF(K39&lt;=0,"Out of stock",IF(K39&lt;=H39,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N39" s="1" t="n"/>
@@ -3271,7 +3272,7 @@
         <v/>
       </c>
       <c r="M40" s="29">
-        <f>IF(B40="","",IF(K40&lt;=0,"✗ Out of stock",IF(K40&lt;=H40,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B40="","",IF(K40&lt;=0,"Out of stock",IF(K40&lt;=H40,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N40" s="1" t="n"/>
@@ -3302,7 +3303,7 @@
         <v/>
       </c>
       <c r="M41" s="29">
-        <f>IF(B41="","",IF(K41&lt;=0,"✗ Out of stock",IF(K41&lt;=H41,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B41="","",IF(K41&lt;=0,"Out of stock",IF(K41&lt;=H41,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N41" s="1" t="n"/>
@@ -3333,7 +3334,7 @@
         <v/>
       </c>
       <c r="M42" s="29">
-        <f>IF(B42="","",IF(K42&lt;=0,"✗ Out of stock",IF(K42&lt;=H42,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B42="","",IF(K42&lt;=0,"Out of stock",IF(K42&lt;=H42,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N42" s="1" t="n"/>
@@ -3364,7 +3365,7 @@
         <v/>
       </c>
       <c r="M43" s="29">
-        <f>IF(B43="","",IF(K43&lt;=0,"✗ Out of stock",IF(K43&lt;=H43,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B43="","",IF(K43&lt;=0,"Out of stock",IF(K43&lt;=H43,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N43" s="1" t="n"/>
@@ -3395,7 +3396,7 @@
         <v/>
       </c>
       <c r="M44" s="29">
-        <f>IF(B44="","",IF(K44&lt;=0,"✗ Out of stock",IF(K44&lt;=H44,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B44="","",IF(K44&lt;=0,"Out of stock",IF(K44&lt;=H44,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N44" s="1" t="n"/>
@@ -3426,7 +3427,7 @@
         <v/>
       </c>
       <c r="M45" s="29">
-        <f>IF(B45="","",IF(K45&lt;=0,"✗ Out of stock",IF(K45&lt;=H45,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B45="","",IF(K45&lt;=0,"Out of stock",IF(K45&lt;=H45,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N45" s="1" t="n"/>
@@ -3457,7 +3458,7 @@
         <v/>
       </c>
       <c r="M46" s="29">
-        <f>IF(B46="","",IF(K46&lt;=0,"✗ Out of stock",IF(K46&lt;=H46,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B46="","",IF(K46&lt;=0,"Out of stock",IF(K46&lt;=H46,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N46" s="1" t="n"/>
@@ -3488,7 +3489,7 @@
         <v/>
       </c>
       <c r="M47" s="29">
-        <f>IF(B47="","",IF(K47&lt;=0,"✗ Out of stock",IF(K47&lt;=H47,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B47="","",IF(K47&lt;=0,"Out of stock",IF(K47&lt;=H47,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N47" s="1" t="n"/>
@@ -3519,7 +3520,7 @@
         <v/>
       </c>
       <c r="M48" s="29">
-        <f>IF(B48="","",IF(K48&lt;=0,"✗ Out of stock",IF(K48&lt;=H48,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B48="","",IF(K48&lt;=0,"Out of stock",IF(K48&lt;=H48,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N48" s="1" t="n"/>
@@ -3550,7 +3551,7 @@
         <v/>
       </c>
       <c r="M49" s="29">
-        <f>IF(B49="","",IF(K49&lt;=0,"✗ Out of stock",IF(K49&lt;=H49,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B49="","",IF(K49&lt;=0,"Out of stock",IF(K49&lt;=H49,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N49" s="1" t="n"/>
@@ -3581,7 +3582,7 @@
         <v/>
       </c>
       <c r="M50" s="29">
-        <f>IF(B50="","",IF(K50&lt;=0,"✗ Out of stock",IF(K50&lt;=H50,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B50="","",IF(K50&lt;=0,"Out of stock",IF(K50&lt;=H50,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N50" s="1" t="n"/>
@@ -3612,7 +3613,7 @@
         <v/>
       </c>
       <c r="M51" s="29">
-        <f>IF(B51="","",IF(K51&lt;=0,"✗ Out of stock",IF(K51&lt;=H51,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B51="","",IF(K51&lt;=0,"Out of stock",IF(K51&lt;=H51,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N51" s="1" t="n"/>
@@ -3643,7 +3644,7 @@
         <v/>
       </c>
       <c r="M52" s="29">
-        <f>IF(B52="","",IF(K52&lt;=0,"✗ Out of stock",IF(K52&lt;=H52,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B52="","",IF(K52&lt;=0,"Out of stock",IF(K52&lt;=H52,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N52" s="1" t="n"/>
@@ -3674,7 +3675,7 @@
         <v/>
       </c>
       <c r="M53" s="29">
-        <f>IF(B53="","",IF(K53&lt;=0,"✗ Out of stock",IF(K53&lt;=H53,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B53="","",IF(K53&lt;=0,"Out of stock",IF(K53&lt;=H53,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N53" s="1" t="n"/>
@@ -3705,7 +3706,7 @@
         <v/>
       </c>
       <c r="M54" s="29">
-        <f>IF(B54="","",IF(K54&lt;=0,"✗ Out of stock",IF(K54&lt;=H54,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B54="","",IF(K54&lt;=0,"Out of stock",IF(K54&lt;=H54,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N54" s="1" t="n"/>
@@ -3736,7 +3737,7 @@
         <v/>
       </c>
       <c r="M55" s="29">
-        <f>IF(B55="","",IF(K55&lt;=0,"✗ Out of stock",IF(K55&lt;=H55,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B55="","",IF(K55&lt;=0,"Out of stock",IF(K55&lt;=H55,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N55" s="1" t="n"/>
@@ -3767,7 +3768,7 @@
         <v/>
       </c>
       <c r="M56" s="29">
-        <f>IF(B56="","",IF(K56&lt;=0,"✗ Out of stock",IF(K56&lt;=H56,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B56="","",IF(K56&lt;=0,"Out of stock",IF(K56&lt;=H56,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N56" s="1" t="n"/>
@@ -3798,7 +3799,7 @@
         <v/>
       </c>
       <c r="M57" s="29">
-        <f>IF(B57="","",IF(K57&lt;=0,"✗ Out of stock",IF(K57&lt;=H57,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B57="","",IF(K57&lt;=0,"Out of stock",IF(K57&lt;=H57,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N57" s="1" t="n"/>
@@ -3829,7 +3830,7 @@
         <v/>
       </c>
       <c r="M58" s="29">
-        <f>IF(B58="","",IF(K58&lt;=0,"✗ Out of stock",IF(K58&lt;=H58,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B58="","",IF(K58&lt;=0,"Out of stock",IF(K58&lt;=H58,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N58" s="1" t="n"/>
@@ -3860,7 +3861,7 @@
         <v/>
       </c>
       <c r="M59" s="29">
-        <f>IF(B59="","",IF(K59&lt;=0,"✗ Out of stock",IF(K59&lt;=H59,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B59="","",IF(K59&lt;=0,"Out of stock",IF(K59&lt;=H59,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N59" s="1" t="n"/>
@@ -3891,7 +3892,7 @@
         <v/>
       </c>
       <c r="M60" s="29">
-        <f>IF(B60="","",IF(K60&lt;=0,"✗ Out of stock",IF(K60&lt;=H60,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B60="","",IF(K60&lt;=0,"Out of stock",IF(K60&lt;=H60,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N60" s="1" t="n"/>
@@ -3922,7 +3923,7 @@
         <v/>
       </c>
       <c r="M61" s="29">
-        <f>IF(B61="","",IF(K61&lt;=0,"✗ Out of stock",IF(K61&lt;=H61,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B61="","",IF(K61&lt;=0,"Out of stock",IF(K61&lt;=H61,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N61" s="1" t="n"/>
@@ -3953,7 +3954,7 @@
         <v/>
       </c>
       <c r="M62" s="29">
-        <f>IF(B62="","",IF(K62&lt;=0,"✗ Out of stock",IF(K62&lt;=H62,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B62="","",IF(K62&lt;=0,"Out of stock",IF(K62&lt;=H62,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N62" s="1" t="n"/>
@@ -3984,7 +3985,7 @@
         <v/>
       </c>
       <c r="M63" s="29">
-        <f>IF(B63="","",IF(K63&lt;=0,"✗ Out of stock",IF(K63&lt;=H63,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B63="","",IF(K63&lt;=0,"Out of stock",IF(K63&lt;=H63,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N63" s="1" t="n"/>
@@ -4015,7 +4016,7 @@
         <v/>
       </c>
       <c r="M64" s="29">
-        <f>IF(B64="","",IF(K64&lt;=0,"✗ Out of stock",IF(K64&lt;=H64,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B64="","",IF(K64&lt;=0,"Out of stock",IF(K64&lt;=H64,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N64" s="1" t="n"/>
@@ -4046,7 +4047,7 @@
         <v/>
       </c>
       <c r="M65" s="29">
-        <f>IF(B65="","",IF(K65&lt;=0,"✗ Out of stock",IF(K65&lt;=H65,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B65="","",IF(K65&lt;=0,"Out of stock",IF(K65&lt;=H65,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N65" s="1" t="n"/>
@@ -4077,7 +4078,7 @@
         <v/>
       </c>
       <c r="M66" s="29">
-        <f>IF(B66="","",IF(K66&lt;=0,"✗ Out of stock",IF(K66&lt;=H66,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B66="","",IF(K66&lt;=0,"Out of stock",IF(K66&lt;=H66,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N66" s="1" t="n"/>
@@ -4108,7 +4109,7 @@
         <v/>
       </c>
       <c r="M67" s="29">
-        <f>IF(B67="","",IF(K67&lt;=0,"✗ Out of stock",IF(K67&lt;=H67,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B67="","",IF(K67&lt;=0,"Out of stock",IF(K67&lt;=H67,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N67" s="1" t="n"/>
@@ -4139,7 +4140,7 @@
         <v/>
       </c>
       <c r="M68" s="29">
-        <f>IF(B68="","",IF(K68&lt;=0,"✗ Out of stock",IF(K68&lt;=H68,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B68="","",IF(K68&lt;=0,"Out of stock",IF(K68&lt;=H68,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N68" s="1" t="n"/>
@@ -4170,7 +4171,7 @@
         <v/>
       </c>
       <c r="M69" s="29">
-        <f>IF(B69="","",IF(K69&lt;=0,"✗ Out of stock",IF(K69&lt;=H69,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B69="","",IF(K69&lt;=0,"Out of stock",IF(K69&lt;=H69,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N69" s="1" t="n"/>
@@ -4201,7 +4202,7 @@
         <v/>
       </c>
       <c r="M70" s="29">
-        <f>IF(B70="","",IF(K70&lt;=0,"✗ Out of stock",IF(K70&lt;=H70,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B70="","",IF(K70&lt;=0,"Out of stock",IF(K70&lt;=H70,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N70" s="1" t="n"/>
@@ -4232,7 +4233,7 @@
         <v/>
       </c>
       <c r="M71" s="29">
-        <f>IF(B71="","",IF(K71&lt;=0,"✗ Out of stock",IF(K71&lt;=H71,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B71="","",IF(K71&lt;=0,"Out of stock",IF(K71&lt;=H71,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N71" s="1" t="n"/>
@@ -4263,7 +4264,7 @@
         <v/>
       </c>
       <c r="M72" s="29">
-        <f>IF(B72="","",IF(K72&lt;=0,"✗ Out of stock",IF(K72&lt;=H72,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B72="","",IF(K72&lt;=0,"Out of stock",IF(K72&lt;=H72,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N72" s="1" t="n"/>
@@ -4294,7 +4295,7 @@
         <v/>
       </c>
       <c r="M73" s="29">
-        <f>IF(B73="","",IF(K73&lt;=0,"✗ Out of stock",IF(K73&lt;=H73,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B73="","",IF(K73&lt;=0,"Out of stock",IF(K73&lt;=H73,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N73" s="1" t="n"/>
@@ -4325,7 +4326,7 @@
         <v/>
       </c>
       <c r="M74" s="29">
-        <f>IF(B74="","",IF(K74&lt;=0,"✗ Out of stock",IF(K74&lt;=H74,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B74="","",IF(K74&lt;=0,"Out of stock",IF(K74&lt;=H74,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N74" s="1" t="n"/>
@@ -4356,7 +4357,7 @@
         <v/>
       </c>
       <c r="M75" s="29">
-        <f>IF(B75="","",IF(K75&lt;=0,"✗ Out of stock",IF(K75&lt;=H75,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B75="","",IF(K75&lt;=0,"Out of stock",IF(K75&lt;=H75,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N75" s="1" t="n"/>
@@ -4387,7 +4388,7 @@
         <v/>
       </c>
       <c r="M76" s="29">
-        <f>IF(B76="","",IF(K76&lt;=0,"✗ Out of stock",IF(K76&lt;=H76,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B76="","",IF(K76&lt;=0,"Out of stock",IF(K76&lt;=H76,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N76" s="1" t="n"/>
@@ -4418,7 +4419,7 @@
         <v/>
       </c>
       <c r="M77" s="29">
-        <f>IF(B77="","",IF(K77&lt;=0,"✗ Out of stock",IF(K77&lt;=H77,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B77="","",IF(K77&lt;=0,"Out of stock",IF(K77&lt;=H77,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N77" s="1" t="n"/>
@@ -4449,7 +4450,7 @@
         <v/>
       </c>
       <c r="M78" s="29">
-        <f>IF(B78="","",IF(K78&lt;=0,"✗ Out of stock",IF(K78&lt;=H78,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B78="","",IF(K78&lt;=0,"Out of stock",IF(K78&lt;=H78,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N78" s="1" t="n"/>
@@ -4480,7 +4481,7 @@
         <v/>
       </c>
       <c r="M79" s="29">
-        <f>IF(B79="","",IF(K79&lt;=0,"✗ Out of stock",IF(K79&lt;=H79,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B79="","",IF(K79&lt;=0,"Out of stock",IF(K79&lt;=H79,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N79" s="1" t="n"/>
@@ -4511,7 +4512,7 @@
         <v/>
       </c>
       <c r="M80" s="29">
-        <f>IF(B80="","",IF(K80&lt;=0,"✗ Out of stock",IF(K80&lt;=H80,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B80="","",IF(K80&lt;=0,"Out of stock",IF(K80&lt;=H80,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N80" s="1" t="n"/>
@@ -4542,7 +4543,7 @@
         <v/>
       </c>
       <c r="M81" s="29">
-        <f>IF(B81="","",IF(K81&lt;=0,"✗ Out of stock",IF(K81&lt;=H81,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B81="","",IF(K81&lt;=0,"Out of stock",IF(K81&lt;=H81,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N81" s="1" t="n"/>
@@ -4573,7 +4574,7 @@
         <v/>
       </c>
       <c r="M82" s="29">
-        <f>IF(B82="","",IF(K82&lt;=0,"✗ Out of stock",IF(K82&lt;=H82,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B82="","",IF(K82&lt;=0,"Out of stock",IF(K82&lt;=H82,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N82" s="1" t="n"/>
@@ -4604,7 +4605,7 @@
         <v/>
       </c>
       <c r="M83" s="29">
-        <f>IF(B83="","",IF(K83&lt;=0,"✗ Out of stock",IF(K83&lt;=H83,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B83="","",IF(K83&lt;=0,"Out of stock",IF(K83&lt;=H83,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N83" s="1" t="n"/>
@@ -4635,7 +4636,7 @@
         <v/>
       </c>
       <c r="M84" s="29">
-        <f>IF(B84="","",IF(K84&lt;=0,"✗ Out of stock",IF(K84&lt;=H84,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B84="","",IF(K84&lt;=0,"Out of stock",IF(K84&lt;=H84,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N84" s="1" t="n"/>
@@ -4666,7 +4667,7 @@
         <v/>
       </c>
       <c r="M85" s="29">
-        <f>IF(B85="","",IF(K85&lt;=0,"✗ Out of stock",IF(K85&lt;=H85,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B85="","",IF(K85&lt;=0,"Out of stock",IF(K85&lt;=H85,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N85" s="1" t="n"/>
@@ -4697,7 +4698,7 @@
         <v/>
       </c>
       <c r="M86" s="29">
-        <f>IF(B86="","",IF(K86&lt;=0,"✗ Out of stock",IF(K86&lt;=H86,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B86="","",IF(K86&lt;=0,"Out of stock",IF(K86&lt;=H86,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N86" s="1" t="n"/>
@@ -4728,7 +4729,7 @@
         <v/>
       </c>
       <c r="M87" s="29">
-        <f>IF(B87="","",IF(K87&lt;=0,"✗ Out of stock",IF(K87&lt;=H87,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B87="","",IF(K87&lt;=0,"Out of stock",IF(K87&lt;=H87,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N87" s="1" t="n"/>
@@ -4759,7 +4760,7 @@
         <v/>
       </c>
       <c r="M88" s="29">
-        <f>IF(B88="","",IF(K88&lt;=0,"✗ Out of stock",IF(K88&lt;=H88,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B88="","",IF(K88&lt;=0,"Out of stock",IF(K88&lt;=H88,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N88" s="1" t="n"/>
@@ -4790,7 +4791,7 @@
         <v/>
       </c>
       <c r="M89" s="29">
-        <f>IF(B89="","",IF(K89&lt;=0,"✗ Out of stock",IF(K89&lt;=H89,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B89="","",IF(K89&lt;=0,"Out of stock",IF(K89&lt;=H89,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N89" s="1" t="n"/>
@@ -4821,7 +4822,7 @@
         <v/>
       </c>
       <c r="M90" s="29">
-        <f>IF(B90="","",IF(K90&lt;=0,"✗ Out of stock",IF(K90&lt;=H90,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B90="","",IF(K90&lt;=0,"Out of stock",IF(K90&lt;=H90,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N90" s="1" t="n"/>
@@ -4852,7 +4853,7 @@
         <v/>
       </c>
       <c r="M91" s="29">
-        <f>IF(B91="","",IF(K91&lt;=0,"✗ Out of stock",IF(K91&lt;=H91,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B91="","",IF(K91&lt;=0,"Out of stock",IF(K91&lt;=H91,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N91" s="1" t="n"/>
@@ -4883,7 +4884,7 @@
         <v/>
       </c>
       <c r="M92" s="29">
-        <f>IF(B92="","",IF(K92&lt;=0,"✗ Out of stock",IF(K92&lt;=H92,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B92="","",IF(K92&lt;=0,"Out of stock",IF(K92&lt;=H92,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N92" s="1" t="n"/>
@@ -4914,7 +4915,7 @@
         <v/>
       </c>
       <c r="M93" s="29">
-        <f>IF(B93="","",IF(K93&lt;=0,"✗ Out of stock",IF(K93&lt;=H93,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B93="","",IF(K93&lt;=0,"Out of stock",IF(K93&lt;=H93,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N93" s="1" t="n"/>
@@ -4945,7 +4946,7 @@
         <v/>
       </c>
       <c r="M94" s="29">
-        <f>IF(B94="","",IF(K94&lt;=0,"✗ Out of stock",IF(K94&lt;=H94,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B94="","",IF(K94&lt;=0,"Out of stock",IF(K94&lt;=H94,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N94" s="1" t="n"/>
@@ -4976,7 +4977,7 @@
         <v/>
       </c>
       <c r="M95" s="29">
-        <f>IF(B95="","",IF(K95&lt;=0,"✗ Out of stock",IF(K95&lt;=H95,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B95="","",IF(K95&lt;=0,"Out of stock",IF(K95&lt;=H95,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N95" s="1" t="n"/>
@@ -5007,7 +5008,7 @@
         <v/>
       </c>
       <c r="M96" s="29">
-        <f>IF(B96="","",IF(K96&lt;=0,"✗ Out of stock",IF(K96&lt;=H96,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B96="","",IF(K96&lt;=0,"Out of stock",IF(K96&lt;=H96,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N96" s="1" t="n"/>
@@ -5038,7 +5039,7 @@
         <v/>
       </c>
       <c r="M97" s="29">
-        <f>IF(B97="","",IF(K97&lt;=0,"✗ Out of stock",IF(K97&lt;=H97,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B97="","",IF(K97&lt;=0,"Out of stock",IF(K97&lt;=H97,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N97" s="1" t="n"/>
@@ -5069,7 +5070,7 @@
         <v/>
       </c>
       <c r="M98" s="29">
-        <f>IF(B98="","",IF(K98&lt;=0,"✗ Out of stock",IF(K98&lt;=H98,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B98="","",IF(K98&lt;=0,"Out of stock",IF(K98&lt;=H98,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N98" s="1" t="n"/>
@@ -5100,7 +5101,7 @@
         <v/>
       </c>
       <c r="M99" s="29">
-        <f>IF(B99="","",IF(K99&lt;=0,"✗ Out of stock",IF(K99&lt;=H99,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B99="","",IF(K99&lt;=0,"Out of stock",IF(K99&lt;=H99,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N99" s="1" t="n"/>
@@ -5131,7 +5132,7 @@
         <v/>
       </c>
       <c r="M100" s="29">
-        <f>IF(B100="","",IF(K100&lt;=0,"✗ Out of stock",IF(K100&lt;=H100,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B100="","",IF(K100&lt;=0,"Out of stock",IF(K100&lt;=H100,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N100" s="1" t="n"/>
@@ -5162,7 +5163,7 @@
         <v/>
       </c>
       <c r="M101" s="29">
-        <f>IF(B101="","",IF(K101&lt;=0,"✗ Out of stock",IF(K101&lt;=H101,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B101="","",IF(K101&lt;=0,"Out of stock",IF(K101&lt;=H101,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N101" s="1" t="n"/>
@@ -5193,7 +5194,7 @@
         <v/>
       </c>
       <c r="M102" s="29">
-        <f>IF(B102="","",IF(K102&lt;=0,"✗ Out of stock",IF(K102&lt;=H102,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B102="","",IF(K102&lt;=0,"Out of stock",IF(K102&lt;=H102,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N102" s="1" t="n"/>
@@ -5224,7 +5225,7 @@
         <v/>
       </c>
       <c r="M103" s="29">
-        <f>IF(B103="","",IF(K103&lt;=0,"✗ Out of stock",IF(K103&lt;=H103,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B103="","",IF(K103&lt;=0,"Out of stock",IF(K103&lt;=H103,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N103" s="1" t="n"/>
@@ -5255,7 +5256,7 @@
         <v/>
       </c>
       <c r="M104" s="29">
-        <f>IF(B104="","",IF(K104&lt;=0,"✗ Out of stock",IF(K104&lt;=H104,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B104="","",IF(K104&lt;=0,"Out of stock",IF(K104&lt;=H104,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N104" s="1" t="n"/>
@@ -5286,7 +5287,7 @@
         <v/>
       </c>
       <c r="M105" s="29">
-        <f>IF(B105="","",IF(K105&lt;=0,"✗ Out of stock",IF(K105&lt;=H105,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B105="","",IF(K105&lt;=0,"Out of stock",IF(K105&lt;=H105,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N105" s="1" t="n"/>
@@ -5317,7 +5318,7 @@
         <v/>
       </c>
       <c r="M106" s="29">
-        <f>IF(B106="","",IF(K106&lt;=0,"✗ Out of stock",IF(K106&lt;=H106,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B106="","",IF(K106&lt;=0,"Out of stock",IF(K106&lt;=H106,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N106" s="1" t="n"/>
@@ -5348,7 +5349,7 @@
         <v/>
       </c>
       <c r="M107" s="29">
-        <f>IF(B107="","",IF(K107&lt;=0,"✗ Out of stock",IF(K107&lt;=H107,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B107="","",IF(K107&lt;=0,"Out of stock",IF(K107&lt;=H107,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N107" s="1" t="n"/>
@@ -5379,7 +5380,7 @@
         <v/>
       </c>
       <c r="M108" s="29">
-        <f>IF(B108="","",IF(K108&lt;=0,"✗ Out of stock",IF(K108&lt;=H108,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B108="","",IF(K108&lt;=0,"Out of stock",IF(K108&lt;=H108,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N108" s="1" t="n"/>
@@ -5410,7 +5411,7 @@
         <v/>
       </c>
       <c r="M109" s="29">
-        <f>IF(B109="","",IF(K109&lt;=0,"✗ Out of stock",IF(K109&lt;=H109,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B109="","",IF(K109&lt;=0,"Out of stock",IF(K109&lt;=H109,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N109" s="1" t="n"/>
@@ -5441,7 +5442,7 @@
         <v/>
       </c>
       <c r="M110" s="29">
-        <f>IF(B110="","",IF(K110&lt;=0,"✗ Out of stock",IF(K110&lt;=H110,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B110="","",IF(K110&lt;=0,"Out of stock",IF(K110&lt;=H110,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N110" s="1" t="n"/>
@@ -5472,7 +5473,7 @@
         <v/>
       </c>
       <c r="M111" s="29">
-        <f>IF(B111="","",IF(K111&lt;=0,"✗ Out of stock",IF(K111&lt;=H111,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B111="","",IF(K111&lt;=0,"Out of stock",IF(K111&lt;=H111,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N111" s="1" t="n"/>
@@ -5503,7 +5504,7 @@
         <v/>
       </c>
       <c r="M112" s="29">
-        <f>IF(B112="","",IF(K112&lt;=0,"✗ Out of stock",IF(K112&lt;=H112,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B112="","",IF(K112&lt;=0,"Out of stock",IF(K112&lt;=H112,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N112" s="1" t="n"/>
@@ -5534,7 +5535,7 @@
         <v/>
       </c>
       <c r="M113" s="29">
-        <f>IF(B113="","",IF(K113&lt;=0,"✗ Out of stock",IF(K113&lt;=H113,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B113="","",IF(K113&lt;=0,"Out of stock",IF(K113&lt;=H113,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N113" s="1" t="n"/>
@@ -5565,7 +5566,7 @@
         <v/>
       </c>
       <c r="M114" s="29">
-        <f>IF(B114="","",IF(K114&lt;=0,"✗ Out of stock",IF(K114&lt;=H114,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B114="","",IF(K114&lt;=0,"Out of stock",IF(K114&lt;=H114,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N114" s="1" t="n"/>
@@ -5596,7 +5597,7 @@
         <v/>
       </c>
       <c r="M115" s="29">
-        <f>IF(B115="","",IF(K115&lt;=0,"✗ Out of stock",IF(K115&lt;=H115,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B115="","",IF(K115&lt;=0,"Out of stock",IF(K115&lt;=H115,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N115" s="1" t="n"/>
@@ -5627,7 +5628,7 @@
         <v/>
       </c>
       <c r="M116" s="29">
-        <f>IF(B116="","",IF(K116&lt;=0,"✗ Out of stock",IF(K116&lt;=H116,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B116="","",IF(K116&lt;=0,"Out of stock",IF(K116&lt;=H116,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N116" s="1" t="n"/>
@@ -5658,7 +5659,7 @@
         <v/>
       </c>
       <c r="M117" s="29">
-        <f>IF(B117="","",IF(K117&lt;=0,"✗ Out of stock",IF(K117&lt;=H117,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B117="","",IF(K117&lt;=0,"Out of stock",IF(K117&lt;=H117,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N117" s="1" t="n"/>
@@ -5689,7 +5690,7 @@
         <v/>
       </c>
       <c r="M118" s="29">
-        <f>IF(B118="","",IF(K118&lt;=0,"✗ Out of stock",IF(K118&lt;=H118,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B118="","",IF(K118&lt;=0,"Out of stock",IF(K118&lt;=H118,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N118" s="1" t="n"/>
@@ -5720,7 +5721,7 @@
         <v/>
       </c>
       <c r="M119" s="29">
-        <f>IF(B119="","",IF(K119&lt;=0,"✗ Out of stock",IF(K119&lt;=H119,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B119="","",IF(K119&lt;=0,"Out of stock",IF(K119&lt;=H119,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N119" s="1" t="n"/>
@@ -5751,7 +5752,7 @@
         <v/>
       </c>
       <c r="M120" s="29">
-        <f>IF(B120="","",IF(K120&lt;=0,"✗ Out of stock",IF(K120&lt;=H120,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B120="","",IF(K120&lt;=0,"Out of stock",IF(K120&lt;=H120,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N120" s="1" t="n"/>
@@ -5782,7 +5783,7 @@
         <v/>
       </c>
       <c r="M121" s="29">
-        <f>IF(B121="","",IF(K121&lt;=0,"✗ Out of stock",IF(K121&lt;=H121,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B121="","",IF(K121&lt;=0,"Out of stock",IF(K121&lt;=H121,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N121" s="1" t="n"/>
@@ -5813,7 +5814,7 @@
         <v/>
       </c>
       <c r="M122" s="29">
-        <f>IF(B122="","",IF(K122&lt;=0,"✗ Out of stock",IF(K122&lt;=H122,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B122="","",IF(K122&lt;=0,"Out of stock",IF(K122&lt;=H122,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N122" s="1" t="n"/>
@@ -5844,7 +5845,7 @@
         <v/>
       </c>
       <c r="M123" s="29">
-        <f>IF(B123="","",IF(K123&lt;=0,"✗ Out of stock",IF(K123&lt;=H123,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B123="","",IF(K123&lt;=0,"Out of stock",IF(K123&lt;=H123,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N123" s="1" t="n"/>
@@ -5875,7 +5876,7 @@
         <v/>
       </c>
       <c r="M124" s="29">
-        <f>IF(B124="","",IF(K124&lt;=0,"✗ Out of stock",IF(K124&lt;=H124,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B124="","",IF(K124&lt;=0,"Out of stock",IF(K124&lt;=H124,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N124" s="1" t="n"/>
@@ -5906,7 +5907,7 @@
         <v/>
       </c>
       <c r="M125" s="29">
-        <f>IF(B125="","",IF(K125&lt;=0,"✗ Out of stock",IF(K125&lt;=H125,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B125="","",IF(K125&lt;=0,"Out of stock",IF(K125&lt;=H125,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N125" s="1" t="n"/>
@@ -5937,7 +5938,7 @@
         <v/>
       </c>
       <c r="M126" s="29">
-        <f>IF(B126="","",IF(K126&lt;=0,"✗ Out of stock",IF(K126&lt;=H126,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B126="","",IF(K126&lt;=0,"Out of stock",IF(K126&lt;=H126,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N126" s="1" t="n"/>
@@ -5968,7 +5969,7 @@
         <v/>
       </c>
       <c r="M127" s="29">
-        <f>IF(B127="","",IF(K127&lt;=0,"✗ Out of stock",IF(K127&lt;=H127,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B127="","",IF(K127&lt;=0,"Out of stock",IF(K127&lt;=H127,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N127" s="1" t="n"/>
@@ -5999,7 +6000,7 @@
         <v/>
       </c>
       <c r="M128" s="29">
-        <f>IF(B128="","",IF(K128&lt;=0,"✗ Out of stock",IF(K128&lt;=H128,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B128="","",IF(K128&lt;=0,"Out of stock",IF(K128&lt;=H128,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N128" s="1" t="n"/>
@@ -6030,7 +6031,7 @@
         <v/>
       </c>
       <c r="M129" s="29">
-        <f>IF(B129="","",IF(K129&lt;=0,"✗ Out of stock",IF(K129&lt;=H129,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B129="","",IF(K129&lt;=0,"Out of stock",IF(K129&lt;=H129,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N129" s="1" t="n"/>
@@ -6061,7 +6062,7 @@
         <v/>
       </c>
       <c r="M130" s="29">
-        <f>IF(B130="","",IF(K130&lt;=0,"✗ Out of stock",IF(K130&lt;=H130,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B130="","",IF(K130&lt;=0,"Out of stock",IF(K130&lt;=H130,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N130" s="1" t="n"/>
@@ -6092,7 +6093,7 @@
         <v/>
       </c>
       <c r="M131" s="29">
-        <f>IF(B131="","",IF(K131&lt;=0,"✗ Out of stock",IF(K131&lt;=H131,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B131="","",IF(K131&lt;=0,"Out of stock",IF(K131&lt;=H131,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N131" s="1" t="n"/>
@@ -6123,7 +6124,7 @@
         <v/>
       </c>
       <c r="M132" s="29">
-        <f>IF(B132="","",IF(K132&lt;=0,"✗ Out of stock",IF(K132&lt;=H132,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B132="","",IF(K132&lt;=0,"Out of stock",IF(K132&lt;=H132,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N132" s="1" t="n"/>
@@ -6154,7 +6155,7 @@
         <v/>
       </c>
       <c r="M133" s="29">
-        <f>IF(B133="","",IF(K133&lt;=0,"✗ Out of stock",IF(K133&lt;=H133,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B133="","",IF(K133&lt;=0,"Out of stock",IF(K133&lt;=H133,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N133" s="1" t="n"/>
@@ -6185,7 +6186,7 @@
         <v/>
       </c>
       <c r="M134" s="29">
-        <f>IF(B134="","",IF(K134&lt;=0,"✗ Out of stock",IF(K134&lt;=H134,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B134="","",IF(K134&lt;=0,"Out of stock",IF(K134&lt;=H134,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N134" s="1" t="n"/>
@@ -6216,7 +6217,7 @@
         <v/>
       </c>
       <c r="M135" s="29">
-        <f>IF(B135="","",IF(K135&lt;=0,"✗ Out of stock",IF(K135&lt;=H135,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B135="","",IF(K135&lt;=0,"Out of stock",IF(K135&lt;=H135,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N135" s="1" t="n"/>
@@ -6247,7 +6248,7 @@
         <v/>
       </c>
       <c r="M136" s="29">
-        <f>IF(B136="","",IF(K136&lt;=0,"✗ Out of stock",IF(K136&lt;=H136,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B136="","",IF(K136&lt;=0,"Out of stock",IF(K136&lt;=H136,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N136" s="1" t="n"/>
@@ -6278,7 +6279,7 @@
         <v/>
       </c>
       <c r="M137" s="29">
-        <f>IF(B137="","",IF(K137&lt;=0,"✗ Out of stock",IF(K137&lt;=H137,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B137="","",IF(K137&lt;=0,"Out of stock",IF(K137&lt;=H137,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N137" s="1" t="n"/>
@@ -6309,7 +6310,7 @@
         <v/>
       </c>
       <c r="M138" s="29">
-        <f>IF(B138="","",IF(K138&lt;=0,"✗ Out of stock",IF(K138&lt;=H138,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B138="","",IF(K138&lt;=0,"Out of stock",IF(K138&lt;=H138,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N138" s="1" t="n"/>
@@ -6340,7 +6341,7 @@
         <v/>
       </c>
       <c r="M139" s="29">
-        <f>IF(B139="","",IF(K139&lt;=0,"✗ Out of stock",IF(K139&lt;=H139,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B139="","",IF(K139&lt;=0,"Out of stock",IF(K139&lt;=H139,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N139" s="1" t="n"/>
@@ -6371,7 +6372,7 @@
         <v/>
       </c>
       <c r="M140" s="29">
-        <f>IF(B140="","",IF(K140&lt;=0,"✗ Out of stock",IF(K140&lt;=H140,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B140="","",IF(K140&lt;=0,"Out of stock",IF(K140&lt;=H140,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N140" s="1" t="n"/>
@@ -6402,7 +6403,7 @@
         <v/>
       </c>
       <c r="M141" s="29">
-        <f>IF(B141="","",IF(K141&lt;=0,"✗ Out of stock",IF(K141&lt;=H141,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B141="","",IF(K141&lt;=0,"Out of stock",IF(K141&lt;=H141,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N141" s="1" t="n"/>
@@ -6433,7 +6434,7 @@
         <v/>
       </c>
       <c r="M142" s="29">
-        <f>IF(B142="","",IF(K142&lt;=0,"✗ Out of stock",IF(K142&lt;=H142,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B142="","",IF(K142&lt;=0,"Out of stock",IF(K142&lt;=H142,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N142" s="1" t="n"/>
@@ -6464,7 +6465,7 @@
         <v/>
       </c>
       <c r="M143" s="29">
-        <f>IF(B143="","",IF(K143&lt;=0,"✗ Out of stock",IF(K143&lt;=H143,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B143="","",IF(K143&lt;=0,"Out of stock",IF(K143&lt;=H143,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N143" s="1" t="n"/>
@@ -6495,7 +6496,7 @@
         <v/>
       </c>
       <c r="M144" s="29">
-        <f>IF(B144="","",IF(K144&lt;=0,"✗ Out of stock",IF(K144&lt;=H144,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B144="","",IF(K144&lt;=0,"Out of stock",IF(K144&lt;=H144,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N144" s="1" t="n"/>
@@ -6526,7 +6527,7 @@
         <v/>
       </c>
       <c r="M145" s="29">
-        <f>IF(B145="","",IF(K145&lt;=0,"✗ Out of stock",IF(K145&lt;=H145,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B145="","",IF(K145&lt;=0,"Out of stock",IF(K145&lt;=H145,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N145" s="1" t="n"/>
@@ -6557,7 +6558,7 @@
         <v/>
       </c>
       <c r="M146" s="29">
-        <f>IF(B146="","",IF(K146&lt;=0,"✗ Out of stock",IF(K146&lt;=H146,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B146="","",IF(K146&lt;=0,"Out of stock",IF(K146&lt;=H146,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N146" s="1" t="n"/>
@@ -6588,7 +6589,7 @@
         <v/>
       </c>
       <c r="M147" s="29">
-        <f>IF(B147="","",IF(K147&lt;=0,"✗ Out of stock",IF(K147&lt;=H147,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B147="","",IF(K147&lt;=0,"Out of stock",IF(K147&lt;=H147,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N147" s="1" t="n"/>
@@ -6619,7 +6620,7 @@
         <v/>
       </c>
       <c r="M148" s="29">
-        <f>IF(B148="","",IF(K148&lt;=0,"✗ Out of stock",IF(K148&lt;=H148,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B148="","",IF(K148&lt;=0,"Out of stock",IF(K148&lt;=H148,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N148" s="1" t="n"/>
@@ -6650,7 +6651,7 @@
         <v/>
       </c>
       <c r="M149" s="29">
-        <f>IF(B149="","",IF(K149&lt;=0,"✗ Out of stock",IF(K149&lt;=H149,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B149="","",IF(K149&lt;=0,"Out of stock",IF(K149&lt;=H149,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N149" s="1" t="n"/>
@@ -6681,7 +6682,7 @@
         <v/>
       </c>
       <c r="M150" s="29">
-        <f>IF(B150="","",IF(K150&lt;=0,"✗ Out of stock",IF(K150&lt;=H150,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B150="","",IF(K150&lt;=0,"Out of stock",IF(K150&lt;=H150,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N150" s="1" t="n"/>
@@ -6712,7 +6713,7 @@
         <v/>
       </c>
       <c r="M151" s="29">
-        <f>IF(B151="","",IF(K151&lt;=0,"✗ Out of stock",IF(K151&lt;=H151,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B151="","",IF(K151&lt;=0,"Out of stock",IF(K151&lt;=H151,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N151" s="1" t="n"/>
@@ -6743,7 +6744,7 @@
         <v/>
       </c>
       <c r="M152" s="29">
-        <f>IF(B152="","",IF(K152&lt;=0,"✗ Out of stock",IF(K152&lt;=H152,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B152="","",IF(K152&lt;=0,"Out of stock",IF(K152&lt;=H152,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N152" s="1" t="n"/>
@@ -6774,7 +6775,7 @@
         <v/>
       </c>
       <c r="M153" s="29">
-        <f>IF(B153="","",IF(K153&lt;=0,"✗ Out of stock",IF(K153&lt;=H153,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B153="","",IF(K153&lt;=0,"Out of stock",IF(K153&lt;=H153,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N153" s="1" t="n"/>
@@ -6805,7 +6806,7 @@
         <v/>
       </c>
       <c r="M154" s="29">
-        <f>IF(B154="","",IF(K154&lt;=0,"✗ Out of stock",IF(K154&lt;=H154,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B154="","",IF(K154&lt;=0,"Out of stock",IF(K154&lt;=H154,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N154" s="1" t="n"/>
@@ -6836,7 +6837,7 @@
         <v/>
       </c>
       <c r="M155" s="29">
-        <f>IF(B155="","",IF(K155&lt;=0,"✗ Out of stock",IF(K155&lt;=H155,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B155="","",IF(K155&lt;=0,"Out of stock",IF(K155&lt;=H155,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N155" s="1" t="n"/>
@@ -6867,7 +6868,7 @@
         <v/>
       </c>
       <c r="M156" s="29">
-        <f>IF(B156="","",IF(K156&lt;=0,"✗ Out of stock",IF(K156&lt;=H156,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B156="","",IF(K156&lt;=0,"Out of stock",IF(K156&lt;=H156,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N156" s="1" t="n"/>
@@ -6898,7 +6899,7 @@
         <v/>
       </c>
       <c r="M157" s="29">
-        <f>IF(B157="","",IF(K157&lt;=0,"✗ Out of stock",IF(K157&lt;=H157,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B157="","",IF(K157&lt;=0,"Out of stock",IF(K157&lt;=H157,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N157" s="1" t="n"/>
@@ -6929,7 +6930,7 @@
         <v/>
       </c>
       <c r="M158" s="29">
-        <f>IF(B158="","",IF(K158&lt;=0,"✗ Out of stock",IF(K158&lt;=H158,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B158="","",IF(K158&lt;=0,"Out of stock",IF(K158&lt;=H158,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N158" s="1" t="n"/>
@@ -6960,7 +6961,7 @@
         <v/>
       </c>
       <c r="M159" s="29">
-        <f>IF(B159="","",IF(K159&lt;=0,"✗ Out of stock",IF(K159&lt;=H159,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B159="","",IF(K159&lt;=0,"Out of stock",IF(K159&lt;=H159,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N159" s="1" t="n"/>
@@ -6991,7 +6992,7 @@
         <v/>
       </c>
       <c r="M160" s="29">
-        <f>IF(B160="","",IF(K160&lt;=0,"✗ Out of stock",IF(K160&lt;=H160,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B160="","",IF(K160&lt;=0,"Out of stock",IF(K160&lt;=H160,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N160" s="1" t="n"/>
@@ -7022,7 +7023,7 @@
         <v/>
       </c>
       <c r="M161" s="29">
-        <f>IF(B161="","",IF(K161&lt;=0,"✗ Out of stock",IF(K161&lt;=H161,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B161="","",IF(K161&lt;=0,"Out of stock",IF(K161&lt;=H161,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N161" s="1" t="n"/>
@@ -7053,7 +7054,7 @@
         <v/>
       </c>
       <c r="M162" s="29">
-        <f>IF(B162="","",IF(K162&lt;=0,"✗ Out of stock",IF(K162&lt;=H162,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B162="","",IF(K162&lt;=0,"Out of stock",IF(K162&lt;=H162,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N162" s="1" t="n"/>
@@ -7084,7 +7085,7 @@
         <v/>
       </c>
       <c r="M163" s="29">
-        <f>IF(B163="","",IF(K163&lt;=0,"✗ Out of stock",IF(K163&lt;=H163,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B163="","",IF(K163&lt;=0,"Out of stock",IF(K163&lt;=H163,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N163" s="1" t="n"/>
@@ -7115,7 +7116,7 @@
         <v/>
       </c>
       <c r="M164" s="29">
-        <f>IF(B164="","",IF(K164&lt;=0,"✗ Out of stock",IF(K164&lt;=H164,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B164="","",IF(K164&lt;=0,"Out of stock",IF(K164&lt;=H164,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N164" s="1" t="n"/>
@@ -7146,7 +7147,7 @@
         <v/>
       </c>
       <c r="M165" s="29">
-        <f>IF(B165="","",IF(K165&lt;=0,"✗ Out of stock",IF(K165&lt;=H165,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B165="","",IF(K165&lt;=0,"Out of stock",IF(K165&lt;=H165,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N165" s="1" t="n"/>
@@ -7177,7 +7178,7 @@
         <v/>
       </c>
       <c r="M166" s="29">
-        <f>IF(B166="","",IF(K166&lt;=0,"✗ Out of stock",IF(K166&lt;=H166,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B166="","",IF(K166&lt;=0,"Out of stock",IF(K166&lt;=H166,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N166" s="1" t="n"/>
@@ -7208,7 +7209,7 @@
         <v/>
       </c>
       <c r="M167" s="29">
-        <f>IF(B167="","",IF(K167&lt;=0,"✗ Out of stock",IF(K167&lt;=H167,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B167="","",IF(K167&lt;=0,"Out of stock",IF(K167&lt;=H167,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N167" s="1" t="n"/>
@@ -7239,7 +7240,7 @@
         <v/>
       </c>
       <c r="M168" s="29">
-        <f>IF(B168="","",IF(K168&lt;=0,"✗ Out of stock",IF(K168&lt;=H168,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B168="","",IF(K168&lt;=0,"Out of stock",IF(K168&lt;=H168,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N168" s="1" t="n"/>
@@ -7270,7 +7271,7 @@
         <v/>
       </c>
       <c r="M169" s="29">
-        <f>IF(B169="","",IF(K169&lt;=0,"✗ Out of stock",IF(K169&lt;=H169,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B169="","",IF(K169&lt;=0,"Out of stock",IF(K169&lt;=H169,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N169" s="1" t="n"/>
@@ -7301,7 +7302,7 @@
         <v/>
       </c>
       <c r="M170" s="29">
-        <f>IF(B170="","",IF(K170&lt;=0,"✗ Out of stock",IF(K170&lt;=H170,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B170="","",IF(K170&lt;=0,"Out of stock",IF(K170&lt;=H170,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N170" s="1" t="n"/>
@@ -7332,7 +7333,7 @@
         <v/>
       </c>
       <c r="M171" s="29">
-        <f>IF(B171="","",IF(K171&lt;=0,"✗ Out of stock",IF(K171&lt;=H171,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B171="","",IF(K171&lt;=0,"Out of stock",IF(K171&lt;=H171,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N171" s="1" t="n"/>
@@ -7363,7 +7364,7 @@
         <v/>
       </c>
       <c r="M172" s="29">
-        <f>IF(B172="","",IF(K172&lt;=0,"✗ Out of stock",IF(K172&lt;=H172,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B172="","",IF(K172&lt;=0,"Out of stock",IF(K172&lt;=H172,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N172" s="1" t="n"/>
@@ -7394,7 +7395,7 @@
         <v/>
       </c>
       <c r="M173" s="29">
-        <f>IF(B173="","",IF(K173&lt;=0,"✗ Out of stock",IF(K173&lt;=H173,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B173="","",IF(K173&lt;=0,"Out of stock",IF(K173&lt;=H173,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N173" s="1" t="n"/>
@@ -7425,7 +7426,7 @@
         <v/>
       </c>
       <c r="M174" s="29">
-        <f>IF(B174="","",IF(K174&lt;=0,"✗ Out of stock",IF(K174&lt;=H174,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B174="","",IF(K174&lt;=0,"Out of stock",IF(K174&lt;=H174,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N174" s="1" t="n"/>
@@ -7456,7 +7457,7 @@
         <v/>
       </c>
       <c r="M175" s="29">
-        <f>IF(B175="","",IF(K175&lt;=0,"✗ Out of stock",IF(K175&lt;=H175,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B175="","",IF(K175&lt;=0,"Out of stock",IF(K175&lt;=H175,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N175" s="1" t="n"/>
@@ -7487,7 +7488,7 @@
         <v/>
       </c>
       <c r="M176" s="29">
-        <f>IF(B176="","",IF(K176&lt;=0,"✗ Out of stock",IF(K176&lt;=H176,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B176="","",IF(K176&lt;=0,"Out of stock",IF(K176&lt;=H176,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N176" s="1" t="n"/>
@@ -7518,7 +7519,7 @@
         <v/>
       </c>
       <c r="M177" s="29">
-        <f>IF(B177="","",IF(K177&lt;=0,"✗ Out of stock",IF(K177&lt;=H177,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B177="","",IF(K177&lt;=0,"Out of stock",IF(K177&lt;=H177,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N177" s="1" t="n"/>
@@ -7549,7 +7550,7 @@
         <v/>
       </c>
       <c r="M178" s="29">
-        <f>IF(B178="","",IF(K178&lt;=0,"✗ Out of stock",IF(K178&lt;=H178,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B178="","",IF(K178&lt;=0,"Out of stock",IF(K178&lt;=H178,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N178" s="1" t="n"/>
@@ -7580,7 +7581,7 @@
         <v/>
       </c>
       <c r="M179" s="29">
-        <f>IF(B179="","",IF(K179&lt;=0,"✗ Out of stock",IF(K179&lt;=H179,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B179="","",IF(K179&lt;=0,"Out of stock",IF(K179&lt;=H179,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N179" s="1" t="n"/>
@@ -7611,7 +7612,7 @@
         <v/>
       </c>
       <c r="M180" s="29">
-        <f>IF(B180="","",IF(K180&lt;=0,"✗ Out of stock",IF(K180&lt;=H180,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B180="","",IF(K180&lt;=0,"Out of stock",IF(K180&lt;=H180,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N180" s="1" t="n"/>
@@ -7642,7 +7643,7 @@
         <v/>
       </c>
       <c r="M181" s="29">
-        <f>IF(B181="","",IF(K181&lt;=0,"✗ Out of stock",IF(K181&lt;=H181,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B181="","",IF(K181&lt;=0,"Out of stock",IF(K181&lt;=H181,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N181" s="1" t="n"/>
@@ -7673,7 +7674,7 @@
         <v/>
       </c>
       <c r="M182" s="29">
-        <f>IF(B182="","",IF(K182&lt;=0,"✗ Out of stock",IF(K182&lt;=H182,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B182="","",IF(K182&lt;=0,"Out of stock",IF(K182&lt;=H182,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N182" s="1" t="n"/>
@@ -7704,7 +7705,7 @@
         <v/>
       </c>
       <c r="M183" s="29">
-        <f>IF(B183="","",IF(K183&lt;=0,"✗ Out of stock",IF(K183&lt;=H183,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B183="","",IF(K183&lt;=0,"Out of stock",IF(K183&lt;=H183,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N183" s="1" t="n"/>
@@ -7735,7 +7736,7 @@
         <v/>
       </c>
       <c r="M184" s="29">
-        <f>IF(B184="","",IF(K184&lt;=0,"✗ Out of stock",IF(K184&lt;=H184,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B184="","",IF(K184&lt;=0,"Out of stock",IF(K184&lt;=H184,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N184" s="1" t="n"/>
@@ -7766,7 +7767,7 @@
         <v/>
       </c>
       <c r="M185" s="29">
-        <f>IF(B185="","",IF(K185&lt;=0,"✗ Out of stock",IF(K185&lt;=H185,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B185="","",IF(K185&lt;=0,"Out of stock",IF(K185&lt;=H185,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N185" s="1" t="n"/>
@@ -7797,7 +7798,7 @@
         <v/>
       </c>
       <c r="M186" s="29">
-        <f>IF(B186="","",IF(K186&lt;=0,"✗ Out of stock",IF(K186&lt;=H186,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B186="","",IF(K186&lt;=0,"Out of stock",IF(K186&lt;=H186,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N186" s="1" t="n"/>
@@ -7828,7 +7829,7 @@
         <v/>
       </c>
       <c r="M187" s="29">
-        <f>IF(B187="","",IF(K187&lt;=0,"✗ Out of stock",IF(K187&lt;=H187,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B187="","",IF(K187&lt;=0,"Out of stock",IF(K187&lt;=H187,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N187" s="1" t="n"/>
@@ -7859,7 +7860,7 @@
         <v/>
       </c>
       <c r="M188" s="29">
-        <f>IF(B188="","",IF(K188&lt;=0,"✗ Out of stock",IF(K188&lt;=H188,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B188="","",IF(K188&lt;=0,"Out of stock",IF(K188&lt;=H188,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N188" s="1" t="n"/>
@@ -7890,7 +7891,7 @@
         <v/>
       </c>
       <c r="M189" s="29">
-        <f>IF(B189="","",IF(K189&lt;=0,"✗ Out of stock",IF(K189&lt;=H189,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B189="","",IF(K189&lt;=0,"Out of stock",IF(K189&lt;=H189,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N189" s="1" t="n"/>
@@ -7921,7 +7922,7 @@
         <v/>
       </c>
       <c r="M190" s="29">
-        <f>IF(B190="","",IF(K190&lt;=0,"✗ Out of stock",IF(K190&lt;=H190,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B190="","",IF(K190&lt;=0,"Out of stock",IF(K190&lt;=H190,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N190" s="1" t="n"/>
@@ -7952,7 +7953,7 @@
         <v/>
       </c>
       <c r="M191" s="29">
-        <f>IF(B191="","",IF(K191&lt;=0,"✗ Out of stock",IF(K191&lt;=H191,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B191="","",IF(K191&lt;=0,"Out of stock",IF(K191&lt;=H191,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N191" s="1" t="n"/>
@@ -7983,7 +7984,7 @@
         <v/>
       </c>
       <c r="M192" s="29">
-        <f>IF(B192="","",IF(K192&lt;=0,"✗ Out of stock",IF(K192&lt;=H192,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B192="","",IF(K192&lt;=0,"Out of stock",IF(K192&lt;=H192,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N192" s="1" t="n"/>
@@ -8014,7 +8015,7 @@
         <v/>
       </c>
       <c r="M193" s="29">
-        <f>IF(B193="","",IF(K193&lt;=0,"✗ Out of stock",IF(K193&lt;=H193,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B193="","",IF(K193&lt;=0,"Out of stock",IF(K193&lt;=H193,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N193" s="1" t="n"/>
@@ -8045,7 +8046,7 @@
         <v/>
       </c>
       <c r="M194" s="29">
-        <f>IF(B194="","",IF(K194&lt;=0,"✗ Out of stock",IF(K194&lt;=H194,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B194="","",IF(K194&lt;=0,"Out of stock",IF(K194&lt;=H194,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N194" s="1" t="n"/>
@@ -8076,7 +8077,7 @@
         <v/>
       </c>
       <c r="M195" s="29">
-        <f>IF(B195="","",IF(K195&lt;=0,"✗ Out of stock",IF(K195&lt;=H195,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B195="","",IF(K195&lt;=0,"Out of stock",IF(K195&lt;=H195,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N195" s="1" t="n"/>
@@ -8107,7 +8108,7 @@
         <v/>
       </c>
       <c r="M196" s="29">
-        <f>IF(B196="","",IF(K196&lt;=0,"✗ Out of stock",IF(K196&lt;=H196,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B196="","",IF(K196&lt;=0,"Out of stock",IF(K196&lt;=H196,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N196" s="1" t="n"/>
@@ -8138,7 +8139,7 @@
         <v/>
       </c>
       <c r="M197" s="29">
-        <f>IF(B197="","",IF(K197&lt;=0,"✗ Out of stock",IF(K197&lt;=H197,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B197="","",IF(K197&lt;=0,"Out of stock",IF(K197&lt;=H197,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N197" s="1" t="n"/>
@@ -8169,7 +8170,7 @@
         <v/>
       </c>
       <c r="M198" s="29">
-        <f>IF(B198="","",IF(K198&lt;=0,"✗ Out of stock",IF(K198&lt;=H198,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B198="","",IF(K198&lt;=0,"Out of stock",IF(K198&lt;=H198,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N198" s="1" t="n"/>
@@ -8200,7 +8201,7 @@
         <v/>
       </c>
       <c r="M199" s="29">
-        <f>IF(B199="","",IF(K199&lt;=0,"✗ Out of stock",IF(K199&lt;=H199,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B199="","",IF(K199&lt;=0,"Out of stock",IF(K199&lt;=H199,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N199" s="1" t="n"/>
@@ -8231,7 +8232,7 @@
         <v/>
       </c>
       <c r="M200" s="29">
-        <f>IF(B200="","",IF(K200&lt;=0,"✗ Out of stock",IF(K200&lt;=H200,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B200="","",IF(K200&lt;=0,"Out of stock",IF(K200&lt;=H200,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N200" s="1" t="n"/>
@@ -8262,7 +8263,7 @@
         <v/>
       </c>
       <c r="M201" s="29">
-        <f>IF(B201="","",IF(K201&lt;=0,"✗ Out of stock",IF(K201&lt;=H201,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B201="","",IF(K201&lt;=0,"Out of stock",IF(K201&lt;=H201,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N201" s="1" t="n"/>
@@ -8293,7 +8294,7 @@
         <v/>
       </c>
       <c r="M202" s="29">
-        <f>IF(B202="","",IF(K202&lt;=0,"✗ Out of stock",IF(K202&lt;=H202,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B202="","",IF(K202&lt;=0,"Out of stock",IF(K202&lt;=H202,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N202" s="1" t="n"/>
@@ -8324,7 +8325,7 @@
         <v/>
       </c>
       <c r="M203" s="29">
-        <f>IF(B203="","",IF(K203&lt;=0,"✗ Out of stock",IF(K203&lt;=H203,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B203="","",IF(K203&lt;=0,"Out of stock",IF(K203&lt;=H203,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N203" s="1" t="n"/>
@@ -8355,7 +8356,7 @@
         <v/>
       </c>
       <c r="M204" s="29">
-        <f>IF(B204="","",IF(K204&lt;=0,"✗ Out of stock",IF(K204&lt;=H204,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B204="","",IF(K204&lt;=0,"Out of stock",IF(K204&lt;=H204,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N204" s="1" t="n"/>
@@ -8386,7 +8387,7 @@
         <v/>
       </c>
       <c r="M205" s="29">
-        <f>IF(B205="","",IF(K205&lt;=0,"✗ Out of stock",IF(K205&lt;=H205,"⚠ Reorder now","✓ OK")))</f>
+        <f>IF(B205="","",IF(K205&lt;=0,"Out of stock",IF(K205&lt;=H205,"Reorder now","OK")))</f>
         <v/>
       </c>
       <c r="N205" s="1" t="n"/>
@@ -8410,13 +8411,13 @@
   </sheetData>
   <conditionalFormatting sqref="M6:M205">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>LEFT($M6,1)="✓"</formula>
+      <formula>$M6="OK"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>LEFT($M6,1)="⚠"</formula>
+      <formula>$M6="Reorder now"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>LEFT($M6,1)="✗"</formula>
+      <formula>$M6="Out of stock"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -44860,7 +44861,7 @@
       <c r="A2" s="1" t="n"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Start here: 10 minutes</t>
+          <t>Start here</t>
         </is>
       </c>
       <c r="C2" s="1" t="n"/>
@@ -44870,7 +44871,7 @@
       <c r="A3" s="1" t="n"/>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Only type in YELLOW cells.</t>
+          <t>Type only in the yellow cells. Everything else is calculated.</t>
         </is>
       </c>
       <c r="C3" s="1" t="n"/>
@@ -44891,7 +44892,7 @@
       </c>
       <c r="C5" s="32" t="inlineStr">
         <is>
-          <t>Products: one line per product: SKU (a short code), name, cost, price, stock today, reorder level.</t>
+          <t>Products: add each product once, with its code, cost, price, stock today and reorder level.</t>
         </is>
       </c>
       <c r="D5" s="1" t="n"/>
@@ -44911,7 +44912,7 @@
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Stock Moves: one line each time stock changes: a Purchase, a Sale, a Return or an Adjustment.</t>
+          <t>Stock Moves: add a line each time stock changes (Purchase, Sale, Return or Adjustment).</t>
         </is>
       </c>
       <c r="D7" s="1" t="n"/>
@@ -44931,7 +44932,7 @@
       </c>
       <c r="C9" s="32" t="inlineStr">
         <is>
-          <t>Adjustment: use a negative quantity for broken, lost or gifted items.</t>
+          <t>Broken, lost or gifted items: add an Adjustment with a negative quantity.</t>
         </is>
       </c>
       <c r="D9" s="1" t="n"/>
@@ -44946,12 +44947,12 @@
       <c r="A11" s="1" t="n"/>
       <c r="B11" s="31" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C11" s="32" t="inlineStr">
         <is>
-          <t>Products shows the stock now and turns orange at the reorder level, red when out of stock.</t>
+          <t>Products then shows the stock you have. Orange means reorder, red means sold out.</t>
         </is>
       </c>
       <c r="D11" s="1" t="n"/>
@@ -44966,12 +44967,12 @@
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="31" t="inlineStr">
         <is>
-          <t>★</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>Dashboard: sales, profit and units per month, stock value, best seller, what to reorder.</t>
+          <t>Dashboard: sales, profit and units for the month you pick, and the value of your stock.</t>
         </is>
       </c>
       <c r="D13" s="1" t="n"/>
@@ -44999,7 +45000,7 @@
       <c r="B17" s="1" t="n"/>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Example products and moves show how it works: delete them and add yours.</t>
+          <t>The example products and moves show how it works. Delete them and add your own.</t>
         </is>
       </c>
       <c r="D17" s="1" t="n"/>
@@ -45015,7 +45016,7 @@
       <c r="B19" s="1" t="n"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Works in Google Sheets and Microsoft Excel. Any currency.</t>
+          <t>Works in Google Sheets and Microsoft Excel, in any currency.</t>
         </is>
       </c>
       <c r="D19" s="1" t="n"/>

</xml_diff>